<commit_message>
Updated Booked hours from yesterday, edited retrospective document, created a Sprint 3 team agreement
</commit_message>
<xml_diff>
--- a/Documentation/Week 8/Booked Hours/Booked_Hours_Christo.xlsx
+++ b/Documentation/Week 8/Booked Hours/Booked_Hours_Christo.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://uniwa-my.sharepoint.com/personal/24432207_student_uwa_edu_au/Documents/UWA - Student/2026_Sem2/CITS3200 - Professional Computing/Project/Repo/CITS3200_Project/Documentation/Week 8/Booked Hours/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="280" documentId="13_ncr:40009_{31A31D98-CA30-574B-8C94-F50C456CB544}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{05F5FEB3-B30A-41BD-A1F7-A6DC25DC3A80}"/>
+  <xr:revisionPtr revIDLastSave="286" documentId="13_ncr:40009_{31A31D98-CA30-574B-8C94-F50C456CB544}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{07A545EE-BE6E-47F8-832F-80F2CD58BF75}"/>
   <bookViews>
     <workbookView xWindow="384" yWindow="384" windowWidth="17280" windowHeight="10008" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="78" uniqueCount="33">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="79" uniqueCount="34">
   <si>
     <t>Wk</t>
   </si>
@@ -147,6 +147,9 @@
   </si>
   <si>
     <t>Retrospective Documentation</t>
+  </si>
+  <si>
+    <t>CycloneDDS Mujoco running documentation</t>
   </si>
 </sst>
 </file>
@@ -378,6 +381,14 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
       <protection locked="0"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" wrapText="1"/>
       <protection locked="0"/>
@@ -396,14 +407,6 @@
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" wrapText="1"/>
       <protection locked="0"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
@@ -841,36 +844,36 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:9" ht="70.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="10" t="s">
+      <c r="A1" s="12" t="s">
         <v>10</v>
       </c>
-      <c r="B1" s="11"/>
-      <c r="C1" s="11"/>
-      <c r="D1" s="11"/>
-      <c r="E1" s="11"/>
-      <c r="F1" s="11"/>
-      <c r="G1" s="11"/>
-      <c r="H1" s="12"/>
+      <c r="B1" s="13"/>
+      <c r="C1" s="13"/>
+      <c r="D1" s="13"/>
+      <c r="E1" s="13"/>
+      <c r="F1" s="13"/>
+      <c r="G1" s="13"/>
+      <c r="H1" s="14"/>
     </row>
     <row r="2" spans="1:9" ht="16.2" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="8" t="s">
         <v>0</v>
       </c>
-      <c r="B2" s="15" t="s">
+      <c r="B2" s="10" t="s">
         <v>1</v>
       </c>
-      <c r="C2" s="16"/>
-      <c r="D2" s="15" t="s">
+      <c r="C2" s="11"/>
+      <c r="D2" s="10" t="s">
         <v>4</v>
       </c>
-      <c r="E2" s="16"/>
+      <c r="E2" s="11"/>
       <c r="F2" s="17" t="s">
         <v>5</v>
       </c>
       <c r="G2" s="8" t="s">
         <v>7</v>
       </c>
-      <c r="H2" s="13" t="s">
+      <c r="H2" s="15" t="s">
         <v>6</v>
       </c>
     </row>
@@ -890,7 +893,7 @@
       </c>
       <c r="F3" s="18"/>
       <c r="G3" s="9"/>
-      <c r="H3" s="14"/>
+      <c r="H3" s="16"/>
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A4" s="1">
@@ -1760,14 +1763,14 @@
       <c r="A31" s="8" t="s">
         <v>0</v>
       </c>
-      <c r="B31" s="15" t="s">
+      <c r="B31" s="10" t="s">
         <v>1</v>
       </c>
-      <c r="C31" s="16"/>
-      <c r="D31" s="15" t="s">
+      <c r="C31" s="11"/>
+      <c r="D31" s="10" t="s">
         <v>4</v>
       </c>
-      <c r="E31" s="16"/>
+      <c r="E31" s="11"/>
       <c r="F31" s="7" t="s">
         <v>5</v>
       </c>
@@ -2125,21 +2128,35 @@
       </c>
     </row>
     <row r="43" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="B43" s="4"/>
-      <c r="C43" s="5"/>
-      <c r="D43" s="4"/>
-      <c r="E43" s="5"/>
-      <c r="G43" s="6" t="str">
+      <c r="A43" s="1">
+        <v>8</v>
+      </c>
+      <c r="B43" s="4">
+        <v>44816</v>
+      </c>
+      <c r="C43" s="5">
+        <v>0.8125</v>
+      </c>
+      <c r="D43" s="4">
+        <v>44816</v>
+      </c>
+      <c r="E43" s="5">
+        <v>0.83333333333333337</v>
+      </c>
+      <c r="F43" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="G43" s="6">
         <f t="shared" si="3"/>
-        <v xml:space="preserve"> </v>
-      </c>
-      <c r="H43" s="1" t="str">
+        <v>0.50000000005820766</v>
+      </c>
+      <c r="H43" s="1">
         <f t="shared" si="4"/>
-        <v xml:space="preserve"> </v>
+        <v>35.749999999883585</v>
       </c>
       <c r="I43" s="1">
         <f t="shared" si="5"/>
-        <v>0</v>
+        <v>0.50000000005820766</v>
       </c>
     </row>
     <row r="44" spans="1:9" x14ac:dyDescent="0.2">
@@ -2509,14 +2526,14 @@
       <c r="A65" s="8" t="s">
         <v>0</v>
       </c>
-      <c r="B65" s="15" t="s">
+      <c r="B65" s="10" t="s">
         <v>1</v>
       </c>
-      <c r="C65" s="16"/>
-      <c r="D65" s="15" t="s">
+      <c r="C65" s="11"/>
+      <c r="D65" s="10" t="s">
         <v>4</v>
       </c>
-      <c r="E65" s="16"/>
+      <c r="E65" s="11"/>
       <c r="F65" s="7" t="s">
         <v>5</v>
       </c>
@@ -3005,14 +3022,14 @@
       <c r="A99" s="8" t="s">
         <v>0</v>
       </c>
-      <c r="B99" s="15" t="s">
+      <c r="B99" s="10" t="s">
         <v>1</v>
       </c>
-      <c r="C99" s="16"/>
-      <c r="D99" s="15" t="s">
+      <c r="C99" s="11"/>
+      <c r="D99" s="10" t="s">
         <v>4</v>
       </c>
-      <c r="E99" s="16"/>
+      <c r="E99" s="11"/>
       <c r="F99" s="7" t="s">
         <v>5</v>
       </c>
@@ -3499,18 +3516,6 @@
     </row>
   </sheetData>
   <mergeCells count="25">
-    <mergeCell ref="H99:H100"/>
-    <mergeCell ref="A99:A100"/>
-    <mergeCell ref="B99:C99"/>
-    <mergeCell ref="D99:E99"/>
-    <mergeCell ref="F99:F100"/>
-    <mergeCell ref="G99:G100"/>
-    <mergeCell ref="G65:G66"/>
-    <mergeCell ref="H65:H66"/>
-    <mergeCell ref="A65:A66"/>
-    <mergeCell ref="B65:C65"/>
-    <mergeCell ref="D65:E65"/>
-    <mergeCell ref="F65:F66"/>
     <mergeCell ref="H31:H32"/>
     <mergeCell ref="G2:G3"/>
     <mergeCell ref="A1:H1"/>
@@ -3524,6 +3529,18 @@
     <mergeCell ref="D31:E31"/>
     <mergeCell ref="F31:F32"/>
     <mergeCell ref="G31:G32"/>
+    <mergeCell ref="G65:G66"/>
+    <mergeCell ref="H65:H66"/>
+    <mergeCell ref="A65:A66"/>
+    <mergeCell ref="B65:C65"/>
+    <mergeCell ref="D65:E65"/>
+    <mergeCell ref="F65:F66"/>
+    <mergeCell ref="H99:H100"/>
+    <mergeCell ref="A99:A100"/>
+    <mergeCell ref="B99:C99"/>
+    <mergeCell ref="D99:E99"/>
+    <mergeCell ref="F99:F100"/>
+    <mergeCell ref="G99:G100"/>
   </mergeCells>
   <phoneticPr fontId="4" type="noConversion"/>
   <pageMargins left="0.74803149606299213" right="0.74803149606299213" top="0.98425196850393704" bottom="0.98425196850393704" header="0.51181102362204722" footer="0.51181102362204722"/>

</xml_diff>